<commit_message>
T6.3 OK : mise à jour tableau tests (NT→OK litige employé)
</commit_message>
<xml_diff>
--- a/docs/tests-manuels-ecoride.xlsx
+++ b/docs/tests-manuels-ecoride.xlsx
@@ -1819,17 +1819,17 @@
       </c>
       <c r="I27" s="7" t="inlineStr">
         <is>
-          <t>Aucun litige actif dans le systeme au moment du test.</t>
-        </is>
-      </c>
-      <c r="J27" s="15" t="inlineStr">
-        <is>
-          <t>NT</t>
+          <t>Litige signalé par le passager, visible dans l'espace employé avec bouton 'Traiter'. Après traitement : flash 'Litige marqué comme traité.' et compteur revient à 0.</t>
+        </is>
+      </c>
+      <c r="J27" s="14" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="K27" s="7" t="inlineStr">
         <is>
-          <t>Pas de litige disponible. Fonctionnalite presente dans le code (espace-employe.php).</t>
+          <t>Fonctionnalité implémentée ce jour (bouton Traiter + handler POST traiter_litige).</t>
         </is>
       </c>
     </row>

</xml_diff>